<commit_message>
feat(db): 13 表口径落地并 psql 实跑通过（4 态房态 / room_block / reservation_price）
- sql/01_schema.sql：13 张表，新增 room_block（维修/停用区间）、reservation_price（逐日成交价格），
  房态改为 4 态（available/cleaning/maintenance/disabled），已预订/入住中由订单推导
- sql/02_constraints.sql：3 条 EXCLUDE（订单重叠、价格方案重叠、封禁区间重叠）、12 触发器、
  2 视图、8 函数；新增跨表校验 fn_check_reservation_block / fn_check_room_block_order（23514）
- sql/03_seed.sql：生成器扩量重生成 —— 30 客户 / 96 预订 / 48 入住 / 96 支付 / 57 服务明细 /
  reservation_price 239 行 / room_block 4 段封禁；room_status_log 降为 11
- sql/04_queries.sql：Q1-Q8 按新口径重写（Q1 排除封禁区间、Q3 扣维修停用房夜、
  Q4 按 actual_checkout_at 归月），实测 Q1 = 35 间
- docs/02 重写为 13 表 / 4 态房态（ER、约束、索引、触发器、B1-B12 边界用例）；
  docs/01、docs/03、docs/05、README、AGENTS.md 全部对齐；新建 docs/页面约定.md
- deliverables：提交件 v2（A4 三页 + xlsx 12x5 + 300dpi 截图，39 项断言 PASS）
- 实跑证据：table_count=13；reservation_price 239；金额不一致 0；overlap_pairs=0；
  DO 块 9 步自检全过（23P01 + 23514）；EXPLAIN 6.264 ms / shared hit=233
</commit_message>
<xml_diff>
--- a/deliverables/第14组_酒店客房预订与入住管理系统_功能清单.xlsx
+++ b/deliverables/第14组_酒店客房预订与入住管理系统_功能清单.xlsx
@@ -97,7 +97,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -470,10 +470,10 @@
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8.5" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="12.5" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -518,7 +518,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="61.6" customHeight="1">
+    <row r="4" ht="62.6" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>F01</t>
@@ -531,7 +531,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>维护房型（名称、床型、面积、容纳人数、标准价、简介）与按日期区间的定价方案。支持新增、修改、停用房型；同一房型在同一日期区间的价格方案不得重叠，价格调整后历史账单按原价保留。</t>
+          <t>维护房型名称、床型、面积、容纳人数、标准价与简介，支持新增、修改及停用；维护按日期区间定价方案，同一房型的价格方案不得重叠，无专项价格时采用标准价。保存订单逐日成交价格，后续调价不修改已确认价格。</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -545,7 +545,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="61.6" customHeight="1">
+    <row r="5" ht="62.6" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>F02</t>
@@ -553,12 +553,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>房间与房态管理</t>
+          <t>房间与基础信息管理</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>维护具体房间（房号唯一、所属房型、楼层、朝向、备注），并管理房态：可用/已预订/入住中/清洁中/维修中/停用。房间停用后不参与可用房查询；房态每次变更写入房态日志，可追溯变更人与时间。</t>
+          <t>维护唯一房号、所属房型、楼层、朝向及备注；管理正常、清洁中、维修中、停用状态，并记录维修、停用的起止日期。房态变更记录操作人与时间。管理员维护员工账号和角色；前台仅办理授权范围内的房态操作。</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -572,7 +572,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="61.6" customHeight="1">
+    <row r="6" ht="62.6" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>F03</t>
@@ -585,156 +585,156 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>客户输入入住日期、离店日期、房型（可选）、入住人数后，系统返回该日期区间内没有预订冲突且房态可用的房间，并按房型汇总剩余数量与区间总价。日期非法（离店早于或等于入住）时给出提示。</t>
+          <t>按入住日期、离店日期、房型（可选）和人数查询，返回区间内无有效订单冲突且无维修、停用冲突的房间，按房型汇总余量及区间报价。校验离店日期晚于入住日期、入住人数不超过房型容量。清洁中房间须完成清洁后才能实际入住。</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
+          <t>客户、前台</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="62.6" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>预订提交</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>客户选定房间及日期后提交预订，校验日期、人数、区间冲突与重复提交；通过后生成唯一预订号，状态为待确认并占用对应日期。保存报价，前台确认时核对成交价格。并发提交由数据库约束与事务控制，冲突时提示重新选择。</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
           <t>客户</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="61.6" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>F04</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>预订提交</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>客户选定房间与日期后提交预订，系统校验：日期区间合法、该房间该区间无其他有效预订、客户无重复提交。校验通过生成唯一预订号，状态为“待确认”；与已有预订冲突时明确提示冲突日期区间。</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>客户</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+    <row r="8" ht="62.6" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>预订管理</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>前台确认或取消预订，按约定到店时限核实未到店订单并释放占用；客户可查看、取消本人尚未入住的预订，查询本人历史入住及消费记录。状态按待确认→已确认→入住中→已完成流转；待确认、已确认可取消，已确认可转未到店；拒绝非法状态变更。</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>客户、前台</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="47.2" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>F05</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>预订管理</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>前台确认、取消预订，并处理“未到店”：未到店与取消的预订释放房间占用；客户可自助取消自己的预订，已入住的预订不允许取消，状态流转不合法时给出提示。</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>客户、前台</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
+    <row r="9" ht="62.6" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>入住与续住办理</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>按预订号或手机号检索订单，核验客户、房间交付状态及日期后办理入住，记录实际入住时间、预计离店日期和押金。散客入住须先建立订单，检查整个区间并保存价格。续住检查新增日期的订单及维修、停用冲突，通过后延长占用区间并保存新增日期价格。</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>前台</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="47.2" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>F06</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>入住办理</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>前台按预订号或客户手机号检索预订，核验后办理入住：生成入住记录、房间房态转为“入住中”、记录实际入住时间与押金，支持无预订的散客直接入住。</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
+    <row r="10" ht="77" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>F07</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>退房与结算</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>记录实际离店时间，按保存的逐日价格与实际计费房晚结算房费，至少计一房晚；登记增值服务项目、数量、单价及费用。结算时抵扣押金，多退少补，保存支付方式及收付款记录。支持提前退房，释放剩余日期占用；超时退房提示前台处理。完成后订单转为已完成，房间转为清洁中。</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>前台</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="61.6" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>F07</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>退房与结算</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>前台办理退房：按实际入住天数与当时适用的房价计算房费，叠加增值服务费用并扣除押金，生成支付记录；房间房态转为“清洁中”。支持提前退房（按实际天数计费）与超时退房提示。</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>前台</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
+    <row r="11" ht="62.6" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>F08</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>房态看板</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>按楼层或房型展示当前运行状态、当日预订与在住信息；预订及在住信息从订单和入住记录获取。支持清洁完成后恢复正常、登记维修区间及结束维修；新增维修、停用安排须检查已有订单，存在冲突时提示先处理订单。</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>前台、管理员</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="61.6" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>F08</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>房态看板</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>以房间为单位的看板视图：按楼层/房型分组展示全部房间的实时房态与当日预订、在住客信息；支持把房间在“清洁中↔可用”“维修中↔可用”之间切换，维修中的房间不参与预订与入住。</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>前台、管理员</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="76" customHeight="1">
+    <row r="12" ht="91.40000000000001" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>F09</t>
@@ -747,7 +747,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>四类统计：①各房型月度入住率（已售房夜/可售房夜）；②月度营业收入（房费+服务费，按支付方式拆分）；③最受欢迎房型 Top N（按订单数与房夜数）；④长期空闲房间（近 90 天无任何预订）与取消率。支持按日期区间与房型筛选。</t>
+          <t>按日期区间及房型筛选：①入住率＝实际入住房晚数÷可售房晚数，可售房晚扣除维修、停用期间，分母为0时显示不适用；②营业收入按退房结算日期汇总房费与服务费，押金不计收入，按支付方式展示净收款；③热门房型分别按有效订单数和实际入住房晚排名；④列出近90天无实际入住的房间，并统计取消率＝已取消订单数÷同期创建订单总数，分母为0时显示不适用。</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -766,7 +766,7 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>